<commit_message>
Daily recap, matchup updates, learning and research 2026-08-23
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-23.xlsx
+++ b/data/k-props/2026-08-23.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="100">
   <si>
     <t>date</t>
   </si>
@@ -145,24 +145,33 @@
     <t>lineup_unweighted_30d_posted</t>
   </si>
   <si>
+    <t>O</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>&lt;6</t>
+  </si>
+  <si>
+    <t>Shane Baz</t>
+  </si>
+  <si>
+    <t>U</t>
+  </si>
+  <si>
+    <t>Kyle Leahy</t>
+  </si>
+  <si>
+    <t>St. Louis Cardinals @ Philadelphia Phillies</t>
+  </si>
+  <si>
+    <t>Cristopher Sánchez</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>&lt;6</t>
-  </si>
-  <si>
-    <t>Shane Baz</t>
-  </si>
-  <si>
-    <t>Kyle Leahy</t>
-  </si>
-  <si>
-    <t>St. Louis Cardinals @ Philadelphia Phillies</t>
-  </si>
-  <si>
-    <t>Cristopher Sánchez</t>
-  </si>
-  <si>
     <t>6-7</t>
   </si>
   <si>
@@ -203,6 +212,9 @@
   </si>
   <si>
     <t>Limited starter</t>
+  </si>
+  <si>
+    <t>L</t>
   </si>
   <si>
     <t>Nolan McLean</t>
@@ -880,17 +892,23 @@
       <c r="Y2">
         <v>1.0574</v>
       </c>
+      <c r="Z2">
+        <v>4</v>
+      </c>
       <c r="AA2" t="s">
         <v>44</v>
       </c>
+      <c r="AB2">
+        <v>0.92</v>
+      </c>
       <c r="AC2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD2">
         <v>4.42</v>
       </c>
       <c r="AE2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF2">
         <v>0.1542</v>
@@ -900,6 +918,18 @@
       </c>
       <c r="AH2">
         <v>0</v>
+      </c>
+      <c r="AI2">
+        <v>-0.42</v>
+      </c>
+      <c r="AJ2">
+        <v>0.42</v>
+      </c>
+      <c r="AK2">
+        <v>-0.42</v>
+      </c>
+      <c r="AL2">
+        <v>0.42</v>
       </c>
       <c r="AM2">
         <v>4.42</v>
@@ -910,7 +940,7 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3">
         <v>4.5</v>
@@ -981,17 +1011,23 @@
       <c r="Y3">
         <v>0.88</v>
       </c>
+      <c r="Z3">
+        <v>3</v>
+      </c>
       <c r="AA3" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB3">
+        <v>-0.92</v>
       </c>
       <c r="AC3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD3">
         <v>3.58</v>
       </c>
       <c r="AE3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF3">
         <v>0.219</v>
@@ -1001,6 +1037,18 @@
       </c>
       <c r="AH3">
         <v>0</v>
+      </c>
+      <c r="AI3">
+        <v>-0.58</v>
+      </c>
+      <c r="AJ3">
+        <v>0.58</v>
+      </c>
+      <c r="AK3">
+        <v>-0.58</v>
+      </c>
+      <c r="AL3">
+        <v>0.58</v>
       </c>
       <c r="AM3">
         <v>3.58</v>
@@ -1011,7 +1059,7 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C4">
         <v>3.5</v>
@@ -1023,7 +1071,7 @@
         <v>132</v>
       </c>
       <c r="F4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G4">
         <v>823421</v>
@@ -1082,17 +1130,23 @@
       <c r="Y4">
         <v>1.0207</v>
       </c>
+      <c r="Z4">
+        <v>4</v>
+      </c>
       <c r="AA4" t="s">
         <v>44</v>
       </c>
+      <c r="AB4">
+        <v>0.7</v>
+      </c>
       <c r="AC4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD4">
         <v>4.2</v>
       </c>
       <c r="AE4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF4">
         <v>0.2352</v>
@@ -1102,6 +1156,18 @@
       </c>
       <c r="AH4">
         <v>0</v>
+      </c>
+      <c r="AI4">
+        <v>-0.2</v>
+      </c>
+      <c r="AJ4">
+        <v>0.2</v>
+      </c>
+      <c r="AK4">
+        <v>-0.2</v>
+      </c>
+      <c r="AL4">
+        <v>0.2</v>
       </c>
       <c r="AM4">
         <v>4.2</v>
@@ -1112,10 +1178,10 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G5">
         <v>823421</v>
@@ -1175,16 +1241,16 @@
         <v>0.9473</v>
       </c>
       <c r="AA5" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC5" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD5">
         <v>6.28</v>
       </c>
       <c r="AE5" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="AF5">
         <v>0.2859</v>
@@ -1204,10 +1270,10 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G6">
         <v>823507</v>
@@ -1267,16 +1333,16 @@
         <v>1.0239</v>
       </c>
       <c r="AA6" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC6" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD6">
         <v>5.99</v>
       </c>
       <c r="AE6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF6">
         <v>0.2193</v>
@@ -1296,10 +1362,10 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G7">
         <v>823507</v>
@@ -1359,16 +1425,16 @@
         <v>0.943</v>
       </c>
       <c r="AA7" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC7" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD7">
         <v>4.2</v>
       </c>
       <c r="AE7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF7">
         <v>0.2504</v>
@@ -1388,7 +1454,7 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C8">
         <v>3.5</v>
@@ -1400,7 +1466,7 @@
         <v>-115</v>
       </c>
       <c r="F8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G8">
         <v>823827</v>
@@ -1459,17 +1525,23 @@
       <c r="Y8">
         <v>0.9665</v>
       </c>
+      <c r="Z8">
+        <v>2</v>
+      </c>
       <c r="AA8" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB8">
+        <v>-0.68</v>
       </c>
       <c r="AC8" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD8">
         <v>2.82</v>
       </c>
       <c r="AE8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF8">
         <v>0.1471</v>
@@ -1479,6 +1551,18 @@
       </c>
       <c r="AH8">
         <v>0</v>
+      </c>
+      <c r="AI8">
+        <v>-0.82</v>
+      </c>
+      <c r="AJ8">
+        <v>0.82</v>
+      </c>
+      <c r="AK8">
+        <v>-0.82</v>
+      </c>
+      <c r="AL8">
+        <v>0.82</v>
       </c>
       <c r="AM8">
         <v>2.82</v>
@@ -1489,16 +1573,16 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G9">
         <v>824071</v>
       </c>
       <c r="H9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I9">
         <v>1.3</v>
@@ -1552,16 +1636,16 @@
         <v>0.88</v>
       </c>
       <c r="AA9" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC9" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD9">
         <v>0.64</v>
       </c>
       <c r="AE9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF9">
         <v>0.1509</v>
@@ -1581,7 +1665,7 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C10">
         <v>2.5</v>
@@ -1593,13 +1677,13 @@
         <v>102</v>
       </c>
       <c r="F10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G10">
         <v>824071</v>
       </c>
       <c r="H10" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I10">
         <v>3</v>
@@ -1652,17 +1736,23 @@
       <c r="Y10">
         <v>0.987</v>
       </c>
+      <c r="Z10">
+        <v>2</v>
+      </c>
       <c r="AA10" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB10">
+        <v>-0.61</v>
       </c>
       <c r="AC10" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD10">
         <v>1.89</v>
       </c>
       <c r="AE10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF10">
         <v>0.177</v>
@@ -1672,6 +1762,18 @@
       </c>
       <c r="AH10">
         <v>0</v>
+      </c>
+      <c r="AI10">
+        <v>0.11</v>
+      </c>
+      <c r="AJ10">
+        <v>0.11</v>
+      </c>
+      <c r="AK10">
+        <v>0.11</v>
+      </c>
+      <c r="AL10">
+        <v>0.11</v>
       </c>
       <c r="AM10">
         <v>1.89</v>
@@ -1682,16 +1784,16 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G11">
         <v>824150</v>
       </c>
       <c r="H11" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I11">
         <v>1.9</v>
@@ -1745,16 +1847,16 @@
         <v>0.9618</v>
       </c>
       <c r="AA11" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC11" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD11">
         <v>1.37</v>
       </c>
       <c r="AE11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF11">
         <v>0.1748</v>
@@ -1774,7 +1876,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C12">
         <v>4.5</v>
@@ -1786,13 +1888,13 @@
         <v>-115</v>
       </c>
       <c r="F12" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G12">
         <v>824150</v>
       </c>
       <c r="H12" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I12">
         <v>3.9</v>
@@ -1845,17 +1947,23 @@
       <c r="Y12">
         <v>1.0766</v>
       </c>
+      <c r="Z12">
+        <v>8</v>
+      </c>
       <c r="AA12" t="s">
         <v>44</v>
       </c>
+      <c r="AB12">
+        <v>-0.89</v>
+      </c>
       <c r="AC12" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="AD12">
         <v>3.61</v>
       </c>
       <c r="AE12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF12">
         <v>0.2069</v>
@@ -1865,6 +1973,18 @@
       </c>
       <c r="AH12">
         <v>0</v>
+      </c>
+      <c r="AI12">
+        <v>4.39</v>
+      </c>
+      <c r="AJ12">
+        <v>4.39</v>
+      </c>
+      <c r="AK12">
+        <v>4.39</v>
+      </c>
+      <c r="AL12">
+        <v>4.39</v>
       </c>
       <c r="AM12">
         <v>3.61</v>
@@ -1875,7 +1995,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C13">
         <v>6.5</v>
@@ -1887,7 +2007,7 @@
         <v>-131</v>
       </c>
       <c r="F13" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="G13">
         <v>824558</v>
@@ -1946,17 +2066,23 @@
       <c r="Y13">
         <v>1.0565</v>
       </c>
+      <c r="Z13">
+        <v>6</v>
+      </c>
       <c r="AA13" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB13">
+        <v>0.49</v>
       </c>
       <c r="AC13" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD13">
         <v>6.99</v>
       </c>
       <c r="AE13" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="AF13">
         <v>0.2496</v>
@@ -1966,6 +2092,18 @@
       </c>
       <c r="AH13">
         <v>0</v>
+      </c>
+      <c r="AI13">
+        <v>-0.99</v>
+      </c>
+      <c r="AJ13">
+        <v>0.99</v>
+      </c>
+      <c r="AK13">
+        <v>-0.99</v>
+      </c>
+      <c r="AL13">
+        <v>0.99</v>
       </c>
       <c r="AM13">
         <v>6.99</v>
@@ -1976,16 +2114,16 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="F14" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="G14">
         <v>824558</v>
       </c>
       <c r="H14" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I14">
         <v>2.1</v>
@@ -2039,16 +2177,16 @@
         <v>0.9312</v>
       </c>
       <c r="AA14" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC14" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD14">
         <v>1.5</v>
       </c>
       <c r="AE14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF14">
         <v>0.2404</v>
@@ -2068,7 +2206,7 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C15">
         <v>4.5</v>
@@ -2080,7 +2218,7 @@
         <v>102</v>
       </c>
       <c r="F15" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G15">
         <v>822856</v>
@@ -2139,17 +2277,23 @@
       <c r="Y15">
         <v>1.0672</v>
       </c>
+      <c r="Z15">
+        <v>4</v>
+      </c>
       <c r="AA15" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB15">
+        <v>0.81</v>
       </c>
       <c r="AC15" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="AD15">
         <v>5.31</v>
       </c>
       <c r="AE15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF15">
         <v>0.2232</v>
@@ -2159,6 +2303,18 @@
       </c>
       <c r="AH15">
         <v>0</v>
+      </c>
+      <c r="AI15">
+        <v>-1.31</v>
+      </c>
+      <c r="AJ15">
+        <v>1.31</v>
+      </c>
+      <c r="AK15">
+        <v>-1.31</v>
+      </c>
+      <c r="AL15">
+        <v>1.31</v>
       </c>
       <c r="AM15">
         <v>5.31</v>
@@ -2169,7 +2325,7 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C16">
         <v>3.5</v>
@@ -2181,7 +2337,7 @@
         <v>120</v>
       </c>
       <c r="F16" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G16">
         <v>822856</v>
@@ -2240,17 +2396,23 @@
       <c r="Y16">
         <v>1.0756</v>
       </c>
+      <c r="Z16">
+        <v>6</v>
+      </c>
       <c r="AA16" t="s">
         <v>44</v>
       </c>
+      <c r="AB16">
+        <v>2.34</v>
+      </c>
       <c r="AC16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD16">
         <v>5.84</v>
       </c>
       <c r="AE16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF16">
         <v>0.1988</v>
@@ -2260,6 +2422,18 @@
       </c>
       <c r="AH16">
         <v>0</v>
+      </c>
+      <c r="AI16">
+        <v>0.16</v>
+      </c>
+      <c r="AJ16">
+        <v>0.16</v>
+      </c>
+      <c r="AK16">
+        <v>0.16</v>
+      </c>
+      <c r="AL16">
+        <v>0.16</v>
       </c>
       <c r="AM16">
         <v>5.84</v>
@@ -2270,7 +2444,7 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C17">
         <v>4.5</v>
@@ -2282,7 +2456,7 @@
         <v>115</v>
       </c>
       <c r="F17" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G17">
         <v>824315</v>
@@ -2341,17 +2515,23 @@
       <c r="Y17">
         <v>1.0231</v>
       </c>
+      <c r="Z17">
+        <v>4</v>
+      </c>
       <c r="AA17" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB17">
+        <v>1.1</v>
       </c>
       <c r="AC17" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="AD17">
         <v>5.6</v>
       </c>
       <c r="AE17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF17">
         <v>0.2121</v>
@@ -2361,6 +2541,18 @@
       </c>
       <c r="AH17">
         <v>0</v>
+      </c>
+      <c r="AI17">
+        <v>-1.6</v>
+      </c>
+      <c r="AJ17">
+        <v>1.6</v>
+      </c>
+      <c r="AK17">
+        <v>-1.6</v>
+      </c>
+      <c r="AL17">
+        <v>1.6</v>
       </c>
       <c r="AM17">
         <v>5.6</v>
@@ -2371,7 +2563,7 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C18">
         <v>2.5</v>
@@ -2383,7 +2575,7 @@
         <v>-110</v>
       </c>
       <c r="F18" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G18">
         <v>824315</v>
@@ -2442,17 +2634,23 @@
       <c r="Y18">
         <v>0.88</v>
       </c>
+      <c r="Z18">
+        <v>2</v>
+      </c>
       <c r="AA18" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB18">
+        <v>-0.29</v>
       </c>
       <c r="AC18" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD18">
         <v>2.21</v>
       </c>
       <c r="AE18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF18">
         <v>0.1367</v>
@@ -2462,6 +2660,18 @@
       </c>
       <c r="AH18">
         <v>0</v>
+      </c>
+      <c r="AI18">
+        <v>-0.21</v>
+      </c>
+      <c r="AJ18">
+        <v>0.21</v>
+      </c>
+      <c r="AK18">
+        <v>-0.21</v>
+      </c>
+      <c r="AL18">
+        <v>0.21</v>
       </c>
       <c r="AM18">
         <v>2.21</v>
@@ -2472,7 +2682,7 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C19">
         <v>4.5</v>
@@ -2484,7 +2694,7 @@
         <v>112</v>
       </c>
       <c r="F19" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G19">
         <v>824720</v>
@@ -2543,17 +2753,23 @@
       <c r="Y19">
         <v>1.0136</v>
       </c>
+      <c r="Z19">
+        <v>6</v>
+      </c>
       <c r="AA19" t="s">
         <v>44</v>
       </c>
+      <c r="AB19">
+        <v>0.95</v>
+      </c>
       <c r="AC19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD19">
         <v>5.45</v>
       </c>
       <c r="AE19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF19">
         <v>0.1953</v>
@@ -2563,6 +2779,18 @@
       </c>
       <c r="AH19">
         <v>0</v>
+      </c>
+      <c r="AI19">
+        <v>0.55</v>
+      </c>
+      <c r="AJ19">
+        <v>0.55</v>
+      </c>
+      <c r="AK19">
+        <v>0.55</v>
+      </c>
+      <c r="AL19">
+        <v>0.55</v>
       </c>
       <c r="AM19">
         <v>5.45</v>
@@ -2573,7 +2801,7 @@
         <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C20">
         <v>2.5</v>
@@ -2585,13 +2813,13 @@
         <v>-179</v>
       </c>
       <c r="F20" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G20">
         <v>823909</v>
       </c>
       <c r="H20" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I20">
         <v>2.3</v>
@@ -2644,17 +2872,23 @@
       <c r="Y20">
         <v>0.9976</v>
       </c>
+      <c r="Z20">
+        <v>1</v>
+      </c>
       <c r="AA20" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB20">
+        <v>0.07</v>
       </c>
       <c r="AC20" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD20">
         <v>2.57</v>
       </c>
       <c r="AE20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF20">
         <v>0.2551</v>
@@ -2664,6 +2898,18 @@
       </c>
       <c r="AH20">
         <v>0</v>
+      </c>
+      <c r="AI20">
+        <v>-1.57</v>
+      </c>
+      <c r="AJ20">
+        <v>1.57</v>
+      </c>
+      <c r="AK20">
+        <v>-1.57</v>
+      </c>
+      <c r="AL20">
+        <v>1.57</v>
       </c>
       <c r="AM20">
         <v>2.57</v>
@@ -2674,7 +2920,7 @@
         <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C21">
         <v>8.5</v>
@@ -2686,7 +2932,7 @@
         <v>-110</v>
       </c>
       <c r="F21" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G21">
         <v>823909</v>
@@ -2745,17 +2991,23 @@
       <c r="Y21">
         <v>1.0405</v>
       </c>
+      <c r="Z21">
+        <v>6</v>
+      </c>
       <c r="AA21" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB21">
+        <v>-1.05</v>
       </c>
       <c r="AC21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD21">
         <v>7.45</v>
       </c>
       <c r="AE21" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AF21">
         <v>0.2902</v>
@@ -2765,6 +3017,18 @@
       </c>
       <c r="AH21">
         <v>0</v>
+      </c>
+      <c r="AI21">
+        <v>-1.45</v>
+      </c>
+      <c r="AJ21">
+        <v>1.45</v>
+      </c>
+      <c r="AK21">
+        <v>-1.45</v>
+      </c>
+      <c r="AL21">
+        <v>1.45</v>
       </c>
       <c r="AM21">
         <v>7.45</v>
@@ -2775,7 +3039,7 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C22">
         <v>5.5</v>
@@ -2787,7 +3051,7 @@
         <v>-106</v>
       </c>
       <c r="F22" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G22">
         <v>823099</v>
@@ -2846,17 +3110,23 @@
       <c r="Y22">
         <v>0.972</v>
       </c>
+      <c r="Z22">
+        <v>4</v>
+      </c>
       <c r="AA22" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB22">
+        <v>-0.27</v>
       </c>
       <c r="AC22" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD22">
         <v>5.23</v>
       </c>
       <c r="AE22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF22">
         <v>0.2611</v>
@@ -2866,6 +3136,18 @@
       </c>
       <c r="AH22">
         <v>0</v>
+      </c>
+      <c r="AI22">
+        <v>-1.23</v>
+      </c>
+      <c r="AJ22">
+        <v>1.23</v>
+      </c>
+      <c r="AK22">
+        <v>-1.23</v>
+      </c>
+      <c r="AL22">
+        <v>1.23</v>
       </c>
       <c r="AM22">
         <v>5.23</v>
@@ -2876,7 +3158,7 @@
         <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C23">
         <v>5.5</v>
@@ -2888,7 +3170,7 @@
         <v>-165</v>
       </c>
       <c r="F23" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G23">
         <v>823099</v>
@@ -2947,17 +3229,23 @@
       <c r="Y23">
         <v>0.941</v>
       </c>
+      <c r="Z23">
+        <v>5</v>
+      </c>
       <c r="AA23" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB23">
+        <v>-0.76</v>
       </c>
       <c r="AC23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD23">
         <v>4.74</v>
       </c>
       <c r="AE23" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF23">
         <v>0.2315</v>
@@ -2967,6 +3255,18 @@
       </c>
       <c r="AH23">
         <v>0</v>
+      </c>
+      <c r="AI23">
+        <v>0.26</v>
+      </c>
+      <c r="AJ23">
+        <v>0.26</v>
+      </c>
+      <c r="AK23">
+        <v>0.26</v>
+      </c>
+      <c r="AL23">
+        <v>0.26</v>
       </c>
       <c r="AM23">
         <v>4.74</v>
@@ -2977,7 +3277,7 @@
         <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C24">
         <v>3.5</v>
@@ -2989,7 +3289,7 @@
         <v>-105</v>
       </c>
       <c r="F24" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G24">
         <v>823258</v>
@@ -3048,17 +3348,23 @@
       <c r="Y24">
         <v>0.9918</v>
       </c>
+      <c r="Z24">
+        <v>3</v>
+      </c>
       <c r="AA24" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB24">
+        <v>-0.72</v>
       </c>
       <c r="AC24" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD24">
         <v>2.78</v>
       </c>
       <c r="AE24" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF24">
         <v>0.1473</v>
@@ -3068,6 +3374,18 @@
       </c>
       <c r="AH24">
         <v>0</v>
+      </c>
+      <c r="AI24">
+        <v>0.22</v>
+      </c>
+      <c r="AJ24">
+        <v>0.22</v>
+      </c>
+      <c r="AK24">
+        <v>0.22</v>
+      </c>
+      <c r="AL24">
+        <v>0.22</v>
       </c>
       <c r="AM24">
         <v>2.78</v>
@@ -3078,7 +3396,7 @@
         <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C25">
         <v>3.5</v>
@@ -3090,7 +3408,7 @@
         <v>118</v>
       </c>
       <c r="F25" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G25">
         <v>823258</v>
@@ -3149,17 +3467,23 @@
       <c r="Y25">
         <v>0.9654</v>
       </c>
+      <c r="Z25">
+        <v>4</v>
+      </c>
       <c r="AA25" t="s">
         <v>44</v>
       </c>
+      <c r="AB25">
+        <v>-0.3</v>
+      </c>
       <c r="AC25" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD25">
         <v>3.2</v>
       </c>
       <c r="AE25" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF25">
         <v>0.1815</v>
@@ -3169,6 +3493,18 @@
       </c>
       <c r="AH25">
         <v>0</v>
+      </c>
+      <c r="AI25">
+        <v>0.8</v>
+      </c>
+      <c r="AJ25">
+        <v>0.8</v>
+      </c>
+      <c r="AK25">
+        <v>0.8</v>
+      </c>
+      <c r="AL25">
+        <v>0.8</v>
       </c>
       <c r="AM25">
         <v>3.2</v>
@@ -3179,7 +3515,7 @@
         <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C26">
         <v>3.5</v>
@@ -3191,7 +3527,7 @@
         <v>-132</v>
       </c>
       <c r="F26" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G26">
         <v>825043</v>
@@ -3250,17 +3586,23 @@
       <c r="Y26">
         <v>0.88</v>
       </c>
+      <c r="Z26">
+        <v>6</v>
+      </c>
       <c r="AA26" t="s">
         <v>44</v>
       </c>
+      <c r="AB26">
+        <v>-0.61</v>
+      </c>
       <c r="AC26" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD26">
         <v>2.89</v>
       </c>
       <c r="AE26" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF26">
         <v>0.1702</v>
@@ -3270,6 +3612,18 @@
       </c>
       <c r="AH26">
         <v>0</v>
+      </c>
+      <c r="AI26">
+        <v>3.11</v>
+      </c>
+      <c r="AJ26">
+        <v>3.11</v>
+      </c>
+      <c r="AK26">
+        <v>3.11</v>
+      </c>
+      <c r="AL26">
+        <v>3.11</v>
       </c>
       <c r="AM26">
         <v>2.89</v>
@@ -3280,7 +3634,7 @@
         <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C27">
         <v>3.5</v>
@@ -3292,13 +3646,13 @@
         <v>134</v>
       </c>
       <c r="F27" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G27">
         <v>825043</v>
       </c>
       <c r="H27" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="I27">
         <v>4.4</v>
@@ -3351,17 +3705,23 @@
       <c r="Y27">
         <v>1.0765</v>
       </c>
+      <c r="Z27">
+        <v>3</v>
+      </c>
       <c r="AA27" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB27">
+        <v>2.05</v>
       </c>
       <c r="AC27" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="AD27">
         <v>5.55</v>
       </c>
       <c r="AE27" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF27">
         <v>0.1666</v>
@@ -3371,6 +3731,18 @@
       </c>
       <c r="AH27">
         <v>0</v>
+      </c>
+      <c r="AI27">
+        <v>-2.55</v>
+      </c>
+      <c r="AJ27">
+        <v>2.55</v>
+      </c>
+      <c r="AK27">
+        <v>-2.55</v>
+      </c>
+      <c r="AL27">
+        <v>2.55</v>
       </c>
       <c r="AM27">
         <v>5.55</v>
@@ -3381,7 +3753,7 @@
         <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C28">
         <v>5.5</v>
@@ -3393,7 +3765,7 @@
         <v>-140</v>
       </c>
       <c r="F28" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G28">
         <v>823745</v>
@@ -3452,17 +3824,23 @@
       <c r="Y28">
         <v>1.04</v>
       </c>
+      <c r="Z28">
+        <v>4</v>
+      </c>
       <c r="AA28" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB28">
+        <v>0.28</v>
       </c>
       <c r="AC28" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AD28">
         <v>5.78</v>
       </c>
       <c r="AE28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF28">
         <v>0.2442</v>
@@ -3472,6 +3850,18 @@
       </c>
       <c r="AH28">
         <v>0</v>
+      </c>
+      <c r="AI28">
+        <v>-1.78</v>
+      </c>
+      <c r="AJ28">
+        <v>1.78</v>
+      </c>
+      <c r="AK28">
+        <v>-1.78</v>
+      </c>
+      <c r="AL28">
+        <v>1.78</v>
       </c>
       <c r="AM28">
         <v>5.78</v>
@@ -3482,7 +3872,7 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C29">
         <v>4.5</v>
@@ -3494,7 +3884,7 @@
         <v>-112</v>
       </c>
       <c r="F29" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G29">
         <v>823745</v>
@@ -3553,17 +3943,23 @@
       <c r="Y29">
         <v>1.0258</v>
       </c>
+      <c r="Z29">
+        <v>5</v>
+      </c>
       <c r="AA29" t="s">
         <v>44</v>
       </c>
+      <c r="AB29">
+        <v>1.6</v>
+      </c>
       <c r="AC29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD29">
         <v>6.1</v>
       </c>
       <c r="AE29" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="AF29">
         <v>0.2438</v>
@@ -3573,6 +3969,18 @@
       </c>
       <c r="AH29">
         <v>0</v>
+      </c>
+      <c r="AI29">
+        <v>-1.1</v>
+      </c>
+      <c r="AJ29">
+        <v>1.1</v>
+      </c>
+      <c r="AK29">
+        <v>-1.1</v>
+      </c>
+      <c r="AL29">
+        <v>1.1</v>
       </c>
       <c r="AM29">
         <v>6.1</v>
@@ -3583,7 +3991,7 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C30">
         <v>6.5</v>
@@ -3595,31 +4003,31 @@
         <v>-108</v>
       </c>
       <c r="F30" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G30" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="H30" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="L30">
         <v>6</v>
       </c>
       <c r="S30" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="V30" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AA30" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC30" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AE30" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:39" x14ac:dyDescent="0.25">
@@ -3627,7 +4035,7 @@
         <v>39</v>
       </c>
       <c r="B31" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C31">
         <v>5.5</v>
@@ -3639,31 +4047,31 @@
         <v>-125</v>
       </c>
       <c r="F31" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G31" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="H31" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="L31">
         <v>6</v>
       </c>
       <c r="S31" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="V31" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AA31" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC31" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AE31" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32" spans="1:39" x14ac:dyDescent="0.25">
@@ -3671,7 +4079,7 @@
         <v>39</v>
       </c>
       <c r="B32" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C32">
         <v>4.5</v>
@@ -3683,31 +4091,31 @@
         <v>114</v>
       </c>
       <c r="F32" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G32" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="H32" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="L32">
         <v>6</v>
       </c>
       <c r="S32" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="V32" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AA32" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC32" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AE32" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="33" spans="1:39" x14ac:dyDescent="0.25">
@@ -3715,7 +4123,7 @@
         <v>39</v>
       </c>
       <c r="B33" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C33">
         <v>4.5</v>
@@ -3727,31 +4135,31 @@
         <v>-162</v>
       </c>
       <c r="F33" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G33" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="H33" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="L33">
         <v>6</v>
       </c>
       <c r="S33" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="V33" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AA33" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC33" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AE33" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
     <row r="34" spans="1:39" x14ac:dyDescent="0.25">
@@ -3759,7 +4167,7 @@
         <v>39</v>
       </c>
       <c r="B34" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C34">
         <v>2.5</v>
@@ -3771,31 +4179,31 @@
         <v>-110</v>
       </c>
       <c r="F34" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G34" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="H34" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="L34">
         <v>3</v>
       </c>
       <c r="S34" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="V34" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AA34" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AC34" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="AE34" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>